<commit_message>
fix: implement copyRowStyleOnly to prevent excel text duplication in merged cells
</commit_message>
<xml_diff>
--- a/public/template_lich_congtac.xlsx
+++ b/public/template_lich_congtac.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A60EA7-640F-48F3-AB5D-A24C3ADCA4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35112FC4-803F-47B4-9AE7-1D3E5582E061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -303,6 +303,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -314,12 +320,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -723,32 +723,32 @@
       <c r="G4" s="17"/>
     </row>
     <row r="5" spans="1:7" ht="16.2" customHeight="1">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" customHeight="1">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
     </row>
     <row r="7" spans="1:7" ht="31.2" customHeight="1">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="4" t="s">
         <v>9</v>
       </c>
@@ -789,24 +789,24 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.8" customHeight="1">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
     </row>
     <row r="10" spans="1:7" ht="83.4" customHeight="1">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="13.8" customHeight="1">
       <c r="A11" s="9"/>

</xml_diff>

<commit_message>
feat: add auto sort button to UI
</commit_message>
<xml_diff>
--- a/public/template_lich_congtac.xlsx
+++ b/public/template_lich_congtac.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35112FC4-803F-47B4-9AE7-1D3E5582E061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29F22B0-CACF-4D99-95C5-3BDBC5B62F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,9 +26,6 @@
     <t>ĐẢNG ỦY XÃ TRÀ BỒNG</t>
   </si>
   <si>
-    <t>{NGAY_BAN_HANH}</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
@@ -81,6 +78,9 @@
   </si>
   <si>
     <t>* Ghi chú: Ngoài thời gian đã bố trí nêu trên, các đồng chí Thường trực Đảng ủy xử lý công việc tại cơ quan hoặc đi công tác cơ sở. Khi có công việc đột xuất, phát sinh sẽ bổ sung Lịch làm việc và thông báo cho các cơ quan, đơn vị liên quan biết</t>
+  </si>
+  <si>
+    <t>Trà Bồng, {NGAY_BAN_HANH}</t>
   </si>
 </sst>
 </file>
@@ -694,7 +694,7 @@
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
       <c r="D2" s="18" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
@@ -702,7 +702,7 @@
     </row>
     <row r="3" spans="1:7" ht="15.6" customHeight="1">
       <c r="A3" s="15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -713,7 +713,7 @@
     </row>
     <row r="4" spans="1:7" ht="15.6" customHeight="1">
       <c r="A4" s="17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -724,7 +724,7 @@
     </row>
     <row r="5" spans="1:7" ht="16.2" customHeight="1">
       <c r="A5" s="21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -735,7 +735,7 @@
     </row>
     <row r="6" spans="1:7" ht="15.6" customHeight="1">
       <c r="A6" s="22" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
@@ -746,46 +746,46 @@
     </row>
     <row r="7" spans="1:7" ht="31.2" customHeight="1">
       <c r="A7" s="23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="31.2" customHeight="1">
       <c r="A8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="G8" s="8" t="s">
         <v>19</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.8" customHeight="1">
@@ -799,7 +799,7 @@
     </row>
     <row r="10" spans="1:7" ht="83.4" customHeight="1">
       <c r="A10" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
@@ -903,7 +903,7 @@
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="A3:C3"/>
   </mergeCells>
-  <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.70866141732283472" right="0.19685039370078741" top="0.78740157480314965" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Optimize UX/UI: Bulk Actions, Global Search, Focus Mode, Performance Analytics & Risk Alerts
</commit_message>
<xml_diff>
--- a/public/template_lich_congtac.xlsx
+++ b/public/template_lich_congtac.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29F22B0-CACF-4D99-95C5-3BDBC5B62F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3686BD80-CCFF-45AE-B12D-AA96B7F2AF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -291,35 +291,35 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -675,80 +675,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.8" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="16" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" ht="15.6" customHeight="1">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
     </row>
     <row r="3" spans="1:7" ht="15.6" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="15.6" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="1:7" ht="16.2" customHeight="1">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" customHeight="1">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" ht="31.2" customHeight="1">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="24"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="4" t="s">
         <v>8</v>
       </c>
@@ -789,24 +789,24 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.8" customHeight="1">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
     </row>
     <row r="10" spans="1:7" ht="83.4" customHeight="1">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="1:7" ht="13.8" customHeight="1">
       <c r="A11" s="9"/>
@@ -890,20 +890,19 @@
       <c r="G19" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A7:B7"/>
+  <mergeCells count="10">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:G1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A7:B7"/>
   </mergeCells>
-  <pageMargins left="0.70866141732283472" right="0.19685039370078741" top="0.78740157480314965" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.70866141732283472" right="0.19685039370078741" top="0.78740157480314965" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>